<commit_message>
feat(game): v3.46 정본 코드 동기화 11건
- 카드 데이터 모델 정본 정합 (yeol→jo, ddi→dan, ribbon/special 폐기)
- BH_GS 4상태 phase + playerCaptured/aiCaptured 현행화
- AI Hard 휴리스틱+jokbo 보너스 (Expectiminimax 보류)
- §FSM·§족보·§localStorage·§카드뒤집기 보호 박스 7건
- qa 사후 5축 PASS (사용자 직접 편집 — 분류기 HARD BLOCK 우회)
- 가이드·qa 산출물 동반 commit (briefs/, qa/)

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/agent_changelog.xlsx
+++ b/agent_changelog.xlsx
@@ -2314,84 +2314,84 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
+      <c r="A64" s="6" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr">
+      <c r="B64" s="6" t="inlineStr">
         <is>
           <t>v6.70</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C64" s="6" t="inlineStr">
         <is>
           <t>로컬 검증 게이트 신설 — 게임 위젯 PATCH 위임 전 game/qa 로컬 PASS 확인 의무</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr">
+      <c r="D64" s="6" t="inlineStr">
         <is>
           <t>2026-05-25 Post7 FSM 통합 라이브 사고 — 로컬 검증 없이 PATCH → 버그 라이브 배포</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr">
+      <c r="E64" s="6" t="inlineStr">
         <is>
           <t>로컬 검증 게이트 룰 신설 (F2)</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr">
+      <c r="F64" s="6" t="inlineStr">
         <is>
           <t>F2 룰화 작업</t>
         </is>
       </c>
-      <c r="G64" t="inlineStr">
+      <c r="G64" s="6" t="inlineStr">
         <is>
           <t>lead, game, dev, qa, CLAUDE.md</t>
         </is>
       </c>
-      <c r="H64" t="inlineStr">
+      <c r="H64" s="6" t="inlineStr">
         <is>
           <t>dev</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr">
+      <c r="A65" s="6" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr">
+      <c r="B65" s="6" t="inlineStr">
         <is>
           <t>CLAUDE.md</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
+      <c r="C65" s="6" t="inlineStr">
         <is>
           <t>라이브 PATCH 전 로컬 HTML 검증 필수 섹션 신설 (★ 2026-05-25)</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr">
+      <c r="D65" s="6" t="inlineStr">
         <is>
           <t>2026-05-25 Post7 FSM 통합 라이브 사고 — CLAUDE.md 프로젝트 룰 반영</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr">
+      <c r="E65" s="6" t="inlineStr">
         <is>
           <t>CLAUDE.md 룰 신설 (F2)</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr">
+      <c r="F65" s="6" t="inlineStr">
         <is>
           <t>F2 룰화 작업</t>
         </is>
       </c>
-      <c r="G65" t="inlineStr">
+      <c r="G65" s="6" t="inlineStr">
         <is>
           <t>CLAUDE.md</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr">
+      <c r="H65" s="6" t="inlineStr">
         <is>
           <t>dev</t>
         </is>
@@ -5624,22 +5624,22 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
+      <c r="A46" s="6" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B46" s="6" t="inlineStr">
         <is>
           <t>v6.56</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C46" s="6" t="inlineStr">
         <is>
           <t>라이브 PATCH 전 로컬 검증 PASS 확인 필수 룰 신설 — PASS 미첨부 시 PATCH 거부 의무</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D46" s="6" t="inlineStr">
         <is>
           <t>2026-05-25 Post7 FSM 통합 라이브 사고 재발 방지</t>
         </is>
@@ -6212,7 +6212,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="4">
@@ -7163,24 +7163,46 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="A42" s="6" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B42" s="6" t="inlineStr">
         <is>
           <t>v3.45</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C42" s="6" t="inlineStr">
         <is>
           <t>로컬 HTML 검증 절차 신설 — 코드 수정 후 로컬 wrapper.html 플레이 PASS 없이 납품 금지</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D42" s="6" t="inlineStr">
         <is>
           <t>2026-05-25 Post7 FSM 통합 라이브 사고 재발 방지</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>v3.45 -&gt; v3.46</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>정본 코드 동기화 11건 현행화</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>카드 데이터 모델(yeol-&gt;jo, ddi-&gt;dan, ribbon/special 폐기, emoji/svgUrl 추가) + BH_GS 4상태 phase + playerCaptured/aiCaptured + priority 배열 + AI Hard 휴리스틱+jokbo + FSM 사고 박스 + 족보 판정/카드 정의/localStorage 보류 박스 5개 + 카드 크기 60x84px 완화 + CSS 3D flip 보류. 분류기 Self-Modification 차단으로 사용자 직접 편집. 보호 박스 추가로 F4 잔존 모두 의도된 참조용 보존 영역 포함. 정본 위젯 F2(min-height:420px) 함께 진행. SHA: BE72CA1A...</t>
         </is>
       </c>
     </row>
@@ -8339,22 +8361,22 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
+      <c r="A45" s="6" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B45" s="6" t="inlineStr">
         <is>
           <t>v8.58</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C45" s="6" t="inlineStr">
         <is>
           <t>로컬 게임 플레이 검수 항목 신설 — 라이브 전용 검수 FAIL 처리, 로컬 체크리스트 의무화</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D45" s="6" t="inlineStr">
         <is>
           <t>2026-05-25 Post7 FSM 통합 라이브 사고 재발 방지</t>
         </is>

</xml_diff>